<commit_message>
feat(pubgen): add GeoJSON Choropleth map charts, decorative cover overlay, and embedded stock maps
</commit_message>
<xml_diff>
--- a/plan/pubgen/samples/DUAL_LANG/BAB_01_2025_ai_translate.xlsx
+++ b/plan/pubgen/samples/DUAL_LANG/BAB_01_2025_ai_translate.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Github\designcraft-pubgen-0.7.X\plan\pubgen\samples\DUAL_LANG\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\GitHub\designcraft-pubgen-07.X\plan\pubgen\samples\DUAL_LANG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCE9135F-D5FC-4FBF-90E8-67AE24FDE533}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55B65853-6798-4AEA-8EA9-74CD4DEEC5D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2505" yWindow="2505" windowWidth="28800" windowHeight="9720" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="COVER" sheetId="7" r:id="rId1"/>
@@ -22,7 +22,8 @@
     <sheet name="R01" sheetId="14" r:id="rId7"/>
     <sheet name="01_01" sheetId="13" r:id="rId8"/>
     <sheet name="03_02" sheetId="16" r:id="rId9"/>
-    <sheet name="note" sheetId="8" r:id="rId10"/>
+    <sheet name="M03_02" sheetId="17" r:id="rId10"/>
+    <sheet name="note" sheetId="8" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_Toc202275224" localSheetId="7">'01_01'!#REF!</definedName>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="104">
   <si>
     <t>Warungbambu</t>
   </si>
@@ -350,6 +351,18 @@
   </si>
   <si>
     <t>images/infografik_01.png</t>
+  </si>
+  <si>
+    <t>map</t>
+  </si>
+  <si>
+    <t>CILAMAYA WETAN</t>
+  </si>
+  <si>
+    <t>data</t>
+  </si>
+  <si>
+    <t>maps\contoh.csv</t>
   </si>
 </sst>
 </file>
@@ -934,6 +947,32 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17BFEEBE-ACB4-41E2-8585-73BA081322F8}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9FF3748-2C15-42F2-916C-09F0CB4E6713}">
   <dimension ref="N1:O11"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>

</xml_diff>